<commit_message>
Update: device control, UDS workbench, DBC parsing, MES precheck and test coverage
</commit_message>
<xml_diff>
--- a/doc/EASY320通道导入模板.xlsx
+++ b/doc/EASY320通道导入模板.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\95403\Desktop\GX_APP刷写设备\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DD1861D-7AE3-4EA0-9D22-0DDC1AA5C011}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42373507-ABD3-459D-9604-840E4212D6F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t>序号</t>
   </si>
@@ -34,21 +34,12 @@
     <t>DO0</t>
   </si>
   <si>
-    <t>平推气缸</t>
-  </si>
-  <si>
     <t>DO1</t>
   </si>
   <si>
-    <t>上升气缸</t>
-  </si>
-  <si>
     <t>DO2</t>
   </si>
   <si>
-    <t>下降气缸</t>
-  </si>
-  <si>
     <t>DO3</t>
   </si>
   <si>
@@ -117,6 +108,34 @@
   </si>
   <si>
     <t>DO27</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>KL30</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>KL15</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>平推气缸(进)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>平推气缸(出)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>抬起</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>下压</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>连接器连接</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -497,129 +516,141 @@
       <c r="A2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
-        <v>3</v>
-      </c>
     </row>
     <row r="3" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>13</v>
+        <v>10</v>
+      </c>
+      <c r="B10" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>14</v>
+        <v>11</v>
+      </c>
+      <c r="B11" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>15</v>
+        <v>12</v>
+      </c>
+      <c r="B12" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>16</v>
+        <v>13</v>
+      </c>
+      <c r="B13" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>17</v>
+        <v>14</v>
+      </c>
+      <c r="B14" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>18</v>
+        <v>15</v>
+      </c>
+      <c r="B15" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>19</v>
+        <v>16</v>
+      </c>
+      <c r="B16" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add relay combination step with UI form and tests
</commit_message>
<xml_diff>
--- a/doc/EASY320通道导入模板.xlsx
+++ b/doc/EASY320通道导入模板.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\95403\Desktop\GX_APP刷写设备\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42373507-ABD3-459D-9604-840E4212D6F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87643ECD-3BE4-43C1-A220-DA9FD2BFA17B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
   <si>
     <t>序号</t>
   </si>
@@ -137,6 +137,60 @@
   <si>
     <t>连接器连接</t>
     <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>DO30</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>DO31</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>DO32</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>DO33</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>DO34</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>DO35</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>DO36</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>DO37</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>温感电阻1</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>温感电阻2</t>
+  </si>
+  <si>
+    <t>温感电阻3</t>
+  </si>
+  <si>
+    <t>温感电阻4</t>
+  </si>
+  <si>
+    <t>温感电阻5</t>
+  </si>
+  <si>
+    <t>温感电阻6</t>
+  </si>
+  <si>
+    <t>温感电阻7</t>
   </si>
 </sst>
 </file>
@@ -497,7 +551,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:B33"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -608,49 +662,110 @@
         <v>27</v>
       </c>
     </row>
-    <row r="17" spans="1:1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B19" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B20" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B21" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B22" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B23" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>25</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>